<commit_message>
Fix NBSP fixture #NAME? via _xlfn.UNICHAR prefix; update QA with real-Excel reproduction results
</commit_message>
<xml_diff>
--- a/fixtures/numbers-stored-as-text-bulk-convert_fixture.xlsx
+++ b/fixtures/numbers-stored-as-text-bulk-convert_fixture.xlsx
@@ -960,7 +960,7 @@
         <v/>
       </c>
       <c r="C4">
-        <f>VALUE(TRIM(SUBSTITUTE(CLEAN(A4),UNICHAR(160)," ")))</f>
+        <f>VALUE(TRIM(SUBSTITUTE(CLEAN(A4),_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -980,7 +980,7 @@
         <v/>
       </c>
       <c r="C5">
-        <f>VALUE(TRIM(SUBSTITUTE(CLEAN(A5),UNICHAR(160)," ")))</f>
+        <f>VALUE(TRIM(SUBSTITUTE(CLEAN(A5),_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1000,7 +1000,7 @@
         <v/>
       </c>
       <c r="C6">
-        <f>VALUE(TRIM(SUBSTITUTE(CLEAN(A6),UNICHAR(160)," ")))</f>
+        <f>VALUE(TRIM(SUBSTITUTE(CLEAN(A6),_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="D6" s="3" t="inlineStr">

</xml_diff>